<commit_message>
feat: implement header aliasing for bulk product import and enhance product detail display for protection plans
</commit_message>
<xml_diff>
--- a/frontend/public/templates/imcorpcart_products_template.xlsx
+++ b/frontend/public/templates/imcorpcart_products_template.xlsx
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="178">
   <si>
     <t>sku</t>
   </si>
@@ -144,10 +144,10 @@
     <t>country_of_origin</t>
   </si>
   <si>
-    <t>protection_plan</t>
-  </si>
-  <si>
-    <t>protection_plan_pct</t>
+    <t>adld</t>
+  </si>
+  <si>
+    <t>adld_pct</t>
   </si>
   <si>
     <t>frequently_bought_skus</t>
@@ -351,7 +351,10 @@
     <t>POINT-WISE and multi-value columns (about_item, in_the_box, spec_rows, image_urls, frequently_bought_skus): put every entry on ONE line separated by a | (pipe). Do NOT press Alt+Enter for a line break inside a cell — this sheet is read as CSV and a line break splits the row.</t>
   </si>
   <si>
-    <t>hsn_code must be 4, 6 or 8 digits (e.g. 8517, 851713 or 85171300). gst_percent accepts "18" or "18%". protection_plan_pct is a % of the EPP price — the rupee amount is calculated for you.</t>
+    <t>hsn_code must be 4, 6 or 8 digits (e.g. 8517, 851713 or 85171300). gst_percent accepts "18" or "18%".</t>
+  </si>
+  <si>
+    <t>ADLD (accidental damage, liquid damage &amp; theft cover): set adld to Applicable and adld_pct to the cover price as a % of the EPP price — the rupee amount is calculated for you and shown to signed-in employees on the product page. The older column names protection_plan / protection_plan_pct still import, so existing sheets keep working.</t>
   </si>
   <si>
     <t>Required columns are tinted blue and show a "Required" note on the header (see the Required column below). The status column only accepts its listed values. Do NOT rename or add symbols to the header row — the importer matches these exact names.</t>
@@ -549,10 +552,10 @@
     <t>Optional · country of manufacture, shown on the product page. The dropdown is only a suggestion — any country name is accepted. e.g. India</t>
   </si>
   <si>
-    <t>products.protection_plan_available (ADLD &amp; theft)</t>
-  </si>
-  <si>
-    <t>Optional · Applicable / Not Applicable — whether an ADLD &amp; theft protection plan is offered on this product. Y / N also accepted.</t>
+    <t>products.protection_plan_available (ADLD &amp; theft cover)</t>
+  </si>
+  <si>
+    <t>Optional · ADLD = accidental damage, liquid damage &amp; theft cover. Applicable / Not Applicable — whether it is offered on this product. Y / N also accepted. Blank leaves the current setting unchanged; Not Applicable switches it off. (The older header protection_plan is still accepted.)</t>
   </si>
   <si>
     <t>pct</t>
@@ -561,7 +564,7 @@
     <t>products.protection_plan_pct</t>
   </si>
   <si>
-    <t>Optional · the plan price as a % of the EPP price (0-100). The rupee amount is calculated for you and shown on the product page. Only used when protection_plan is Applicable. e.g. 7.5</t>
+    <t>Optional · the ADLD cover price as a % of the EPP price (0-100). The rupee amount is calculated for you and shown to signed-in employees on the product page. Only used when adld is Applicable. e.g. 7.5 (The older header protection_plan_pct is still accepted.)</t>
   </si>
   <si>
     <t>products.frequently_bought_skus → the "Frequently bought together" shelf</t>
@@ -11952,7 +11955,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -12088,49 +12091,41 @@
       <c r="D15" s="10"/>
       <c r="E15" s="10"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="B18" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="C18" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="D18" s="11" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>0</v>
-      </c>
-      <c r="B18" s="12" t="s">
+      <c r="E18" s="11" t="s">
         <v>109</v>
-      </c>
-      <c r="C18" t="s">
-        <v>110</v>
-      </c>
-      <c r="D18" t="s">
-        <v>111</v>
-      </c>
-      <c r="E18" s="13" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C19" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D19" t="s">
         <v>112</v>
@@ -12141,16 +12136,16 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>2</v>
-      </c>
-      <c r="B20" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="C20" t="s">
+        <v>111</v>
+      </c>
+      <c r="D20" t="s">
         <v>113</v>
-      </c>
-      <c r="C20" t="s">
-        <v>110</v>
-      </c>
-      <c r="D20" t="s">
-        <v>114</v>
       </c>
       <c r="E20" s="13" t="s">
         <v>67</v>
@@ -12158,13 +12153,13 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B21" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C21" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D21" t="s">
         <v>115</v>
@@ -12175,516 +12170,533 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>4</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>109</v>
+        <v>3</v>
+      </c>
+      <c r="B22" t="s">
+        <v>114</v>
       </c>
       <c r="C22" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D22" t="s">
         <v>116</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>117</v>
+        <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>5</v>
-      </c>
-      <c r="B23" t="s">
-        <v>113</v>
+        <v>4</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>110</v>
       </c>
       <c r="C23" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D23" t="s">
+        <v>117</v>
+      </c>
+      <c r="E23" s="13" t="s">
         <v>118</v>
-      </c>
-      <c r="E23" s="13" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B24" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C24" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D24" t="s">
+        <v>119</v>
+      </c>
+      <c r="E24" s="13" t="s">
         <v>120</v>
-      </c>
-      <c r="E24" s="13" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B25" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C25" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D25" t="s">
+        <v>121</v>
+      </c>
+      <c r="E25" s="13" t="s">
         <v>122</v>
-      </c>
-      <c r="E25" s="13" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B26" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C26" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D26" t="s">
+        <v>123</v>
+      </c>
+      <c r="E26" s="13" t="s">
         <v>124</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B27" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C27" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D27" t="s">
+        <v>125</v>
+      </c>
+      <c r="E27" s="13" t="s">
         <v>126</v>
-      </c>
-      <c r="E27" s="13" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B28" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C28" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D28" t="s">
+        <v>127</v>
+      </c>
+      <c r="E28" s="13" t="s">
         <v>128</v>
-      </c>
-      <c r="E28" s="13" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D29" t="s">
+        <v>129</v>
+      </c>
+      <c r="E29" s="13" t="s">
         <v>130</v>
-      </c>
-      <c r="E29" s="13" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B30" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C30" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D30" t="s">
+        <v>131</v>
+      </c>
+      <c r="E30" s="13" t="s">
         <v>132</v>
-      </c>
-      <c r="E30" s="13" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B31" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C31" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D31" t="s">
+        <v>133</v>
+      </c>
+      <c r="E31" s="13" t="s">
         <v>134</v>
-      </c>
-      <c r="E31" s="13" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B32" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C32" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D32" t="s">
+        <v>135</v>
+      </c>
+      <c r="E32" s="13" t="s">
         <v>136</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B33" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C33" t="s">
+        <v>111</v>
+      </c>
+      <c r="D33" t="s">
+        <v>137</v>
+      </c>
+      <c r="E33" s="13" t="s">
         <v>138</v>
-      </c>
-      <c r="D33" t="s">
-        <v>139</v>
-      </c>
-      <c r="E33" s="13" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B34" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C34" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D34" t="s">
+        <v>140</v>
+      </c>
+      <c r="E34" s="13" t="s">
         <v>141</v>
-      </c>
-      <c r="E34" s="13" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>17</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>109</v>
+        <v>16</v>
+      </c>
+      <c r="B35" t="s">
+        <v>114</v>
       </c>
       <c r="C35" t="s">
+        <v>139</v>
+      </c>
+      <c r="D35" t="s">
+        <v>142</v>
+      </c>
+      <c r="E35" s="13" t="s">
         <v>143</v>
-      </c>
-      <c r="D35" t="s">
-        <v>144</v>
-      </c>
-      <c r="E35" s="13" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>18</v>
-      </c>
-      <c r="B36" t="s">
-        <v>113</v>
+        <v>17</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>110</v>
       </c>
       <c r="C36" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D36" t="s">
+        <v>145</v>
+      </c>
+      <c r="E36" s="13" t="s">
         <v>146</v>
-      </c>
-      <c r="E36" s="13" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B37" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C37" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D37" t="s">
         <v>147</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B38" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C38" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D38" t="s">
+        <v>148</v>
+      </c>
+      <c r="E38" s="13" t="s">
         <v>149</v>
-      </c>
-      <c r="E38" s="13" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B39" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C39" t="s">
-        <v>110</v>
+        <v>144</v>
       </c>
       <c r="D39" t="s">
+        <v>150</v>
+      </c>
+      <c r="E39" s="13" t="s">
         <v>151</v>
-      </c>
-      <c r="E39" s="13" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B40" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C40" t="s">
-        <v>143</v>
+        <v>111</v>
       </c>
       <c r="D40" t="s">
+        <v>152</v>
+      </c>
+      <c r="E40" s="13" t="s">
         <v>153</v>
-      </c>
-      <c r="E40" s="13" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B41" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C41" t="s">
-        <v>110</v>
+        <v>144</v>
       </c>
       <c r="D41" t="s">
+        <v>154</v>
+      </c>
+      <c r="E41" s="13" t="s">
         <v>155</v>
-      </c>
-      <c r="E41" s="13" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B42" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C42" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D42" t="s">
+        <v>156</v>
+      </c>
+      <c r="E42" s="13" t="s">
         <v>157</v>
-      </c>
-      <c r="E42" s="13" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B43" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C43" t="s">
-        <v>138</v>
+        <v>111</v>
       </c>
       <c r="D43" t="s">
+        <v>158</v>
+      </c>
+      <c r="E43" s="13" t="s">
         <v>159</v>
-      </c>
-      <c r="E43" s="13" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B44" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C44" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D44" t="s">
+        <v>160</v>
+      </c>
+      <c r="E44" s="13" t="s">
         <v>161</v>
-      </c>
-      <c r="E44" s="13" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B45" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C45" t="s">
+        <v>139</v>
+      </c>
+      <c r="D45" t="s">
+        <v>162</v>
+      </c>
+      <c r="E45" s="13" t="s">
         <v>163</v>
-      </c>
-      <c r="D45" t="s">
-        <v>164</v>
-      </c>
-      <c r="E45" s="13" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B46" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C46" t="s">
-        <v>110</v>
+        <v>164</v>
       </c>
       <c r="D46" t="s">
+        <v>165</v>
+      </c>
+      <c r="E46" s="13" t="s">
         <v>166</v>
-      </c>
-      <c r="E46" s="13" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B47" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C47" t="s">
-        <v>138</v>
+        <v>111</v>
       </c>
       <c r="D47" t="s">
+        <v>167</v>
+      </c>
+      <c r="E47" s="13" t="s">
         <v>168</v>
-      </c>
-      <c r="E47" s="13" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>30</v>
-      </c>
-      <c r="B48" s="12" t="s">
-        <v>109</v>
+        <v>29</v>
+      </c>
+      <c r="B48" t="s">
+        <v>114</v>
       </c>
       <c r="C48" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D48" t="s">
+        <v>169</v>
+      </c>
+      <c r="E48" s="13" t="s">
         <v>170</v>
-      </c>
-      <c r="E48" s="13" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>31</v>
-      </c>
-      <c r="B49" t="s">
-        <v>113</v>
+        <v>30</v>
+      </c>
+      <c r="B49" s="12" t="s">
+        <v>110</v>
       </c>
       <c r="C49" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D49" t="s">
         <v>171</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>32</v>
-      </c>
-      <c r="B50" s="12" t="s">
-        <v>109</v>
+        <v>31</v>
+      </c>
+      <c r="B50" t="s">
+        <v>114</v>
       </c>
       <c r="C50" t="s">
+        <v>144</v>
+      </c>
+      <c r="D50" t="s">
         <v>172</v>
       </c>
-      <c r="D50" t="s">
-        <v>173</v>
-      </c>
       <c r="E50" s="13" t="s">
-        <v>174</v>
+        <v>146</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>32</v>
+      </c>
+      <c r="B51" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="C51" t="s">
+        <v>173</v>
+      </c>
+      <c r="D51" t="s">
+        <v>174</v>
+      </c>
+      <c r="E51" s="13" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>33</v>
       </c>
-      <c r="B51" t="s">
-        <v>113</v>
-      </c>
-      <c r="C51" t="s">
-        <v>110</v>
-      </c>
-      <c r="D51" t="s">
-        <v>175</v>
-      </c>
-      <c r="E51" s="13" t="s">
+      <c r="B52" t="s">
+        <v>114</v>
+      </c>
+      <c r="C52" t="s">
+        <v>111</v>
+      </c>
+      <c r="D52" t="s">
         <v>176</v>
       </c>
+      <c r="E52" s="13" t="s">
+        <v>177</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A4:E4"/>
@@ -12699,6 +12711,7 @@
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A16:E16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: enhance order management and reporting features
- Added new CSS styles for order table in Partners module to improve layout and readability.
- Refactored Pincodes component to utilize centralized courier options.
- Exported PERIODS constant in ReportFilters for reuse in other components.
- Introduced Shipment_Status_Matcher.xlsx for tracking shipment statuses.
- Modified orders table to include new columns for invoice number and timestamp.
- Updated CourierCode enum with new values and added corresponding courier rows.
- Implemented automatic proof-of-delivery fetch state in shipments table.
- Created shopStatusLabel utility to map order statuses to user-friendly labels.
- Defined SHOP_STATUS_TONE for visual representation of order statuses.
- Added shopStatusBucket function to categorize order statuses for UI display.
- Mapped shipment event codes to user-friendly labels for tracking events.
</commit_message>
<xml_diff>
--- a/frontend/public/templates/imcorpcart_products_template.xlsx
+++ b/frontend/public/templates/imcorpcart_products_template.xlsx
@@ -11950,11 +11950,11 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" error="Pick one of: Applicable, Not Applicable" sqref="AA2:AA800">
       <formula1>"Applicable,Not Applicable"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" error="Pick one of: BLUEDART, DELHIVERY, DTDC, EKART, INDIA_POST" sqref="AD10:AD800">
-      <formula1>"BLUEDART,DELHIVERY,DTDC,EKART,INDIA_POST"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" error="Pick one of: BLUEDART, DELHIVERY, DTDC, EKART, INDIA_POST, GATI, CRITICALLOG, JAYDEEP, MOVIN, DELHIVERY_B2B" sqref="AD10:AD800">
+      <formula1>"BLUEDART,DELHIVERY,DTDC,EKART,INDIA_POST,GATI,CRITICALLOG,JAYDEEP,MOVIN,DELHIVERY_B2B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" error="Pick one of: BLUEDART, DELHIVERY, DTDC, EKART, INDIA_POST" sqref="AD2:AD800">
-      <formula1>"BLUEDART,DELHIVERY,DTDC,EKART,INDIA_POST"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" error="Pick one of: BLUEDART, DELHIVERY, DTDC, EKART, INDIA_POST, GATI, CRITICALLOG, JAYDEEP, MOVIN, DELHIVERY_B2B" sqref="AD2:AD800">
+      <formula1>"BLUEDART,DELHIVERY,DTDC,EKART,INDIA_POST,GATI,CRITICALLOG,JAYDEEP,MOVIN,DELHIVERY_B2B"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" error="Pick one of: APEX, DP, SURFACE" sqref="AE10:AE800">
       <formula1>"APEX,DP,SURFACE"</formula1>

</xml_diff>